<commit_message>
product backlog & sprint 1 backlog updated
</commit_message>
<xml_diff>
--- a/docs/scrum/sprint-backlogs/sprint-1.xlsx
+++ b/docs/scrum/sprint-backlogs/sprint-1.xlsx
@@ -28,19 +28,19 @@
     <t xml:space="preserve">Sprint Backlog</t>
   </si>
   <si>
-    <t xml:space="preserve">Ainullah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set up Node.js project</t>
+    <t xml:space="preserve">Reza Panahi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set up Node.js </t>
   </si>
   <si>
     <t xml:space="preserve">Set up Neon PostgreSQL database</t>
   </si>
   <si>
-    <t xml:space="preserve">Configure Sequelize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reza</t>
+    <t xml:space="preserve">Configure Sequelize &amp; Env</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auinullha Amery </t>
   </si>
   <si>
     <t xml:space="preserve">Create Coin model</t>
@@ -49,19 +49,19 @@
     <t xml:space="preserve">Create Email model</t>
   </si>
   <si>
-    <t xml:space="preserve">Create Coin CRUD scripts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mahfuz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create Email CRUD scripts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add Zod validation for Coin scripts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add Zod validation for Email scripts</t>
+    <t xml:space="preserve">Ghulam Mahfoz Osmani </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrate CoinLore REST API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write Coin service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrate Gmail SMTP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write Email services</t>
   </si>
 </sst>
 </file>
@@ -71,11 +71,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Tahoma"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -95,24 +96,58 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF993300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8000"/>
+        <bgColor rgb="FFFF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFBF00"/>
+        <bgColor rgb="FFFF8000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -120,6 +155,13 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -146,21 +188,41 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -172,6 +234,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFBF00"/>
+      <rgbColor rgb="FFFF8000"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -289,88 +411,87 @@
   <dimension ref="K1:L10"/>
   <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="4.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="30.5"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="29.39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K5" s="2" t="s">
+    <row r="5" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K6" s="2" t="s">
+    <row r="6" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L7" s="3" t="s">
+    <row r="7" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K7" s="5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K8" s="2" t="s">
+      <c r="L7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="3" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L8" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L9" s="3" t="s">
+    <row r="9" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L9" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L10" s="3" t="s">
+    <row r="10" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L10" s="7" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>